<commit_message>
Add updated analysis files
</commit_message>
<xml_diff>
--- a/output/tables/celltype_development_tables.xlsx
+++ b/output/tables/celltype_development_tables.xlsx
@@ -12,14 +12,14 @@
     <sheet name="dropseq_dev" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="multiple_sclerosis_cell_type" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="multiple_sclerosis_dev" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="glioma_cell_type" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="glioma_dev" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="dmg_cell_type" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="dmg_dev" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t xml:space="preserve">sample_id</t>
   </si>
@@ -27,63 +27,63 @@
     <t xml:space="preserve">dev.group</t>
   </si>
   <si>
-    <t xml:space="preserve">ROBO2 Ependymal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLIT2 Ependymal</t>
+    <t xml:space="preserve">Ependymal</t>
   </si>
   <si>
     <t xml:space="preserve">Radial Glia</t>
   </si>
   <si>
-    <t xml:space="preserve">Transit Amplifying Cell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAX3 Neuroblast</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAX3 Neuron</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOXB3 Neuroblast</t>
+    <t xml:space="preserve">Astrocyte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intermediate Proliferative Cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAX6+ NEUROD1+ Neuroblast</t>
   </si>
   <si>
     <t xml:space="preserve">Neuron</t>
   </si>
   <si>
+    <t xml:space="preserve">PAX6+ HOXB3+ Neuroblast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fetal Neuronal Progenitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fetal COP</t>
+  </si>
+  <si>
     <t xml:space="preserve">OPC</t>
   </si>
   <si>
-    <t xml:space="preserve">Fetal COP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Early Oligo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oligo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Astrocyte</t>
+    <t xml:space="preserve">Early OL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postnatal Glial Progenitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endothelial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pericyte</t>
   </si>
   <si>
     <t xml:space="preserve">Mesenchymal</t>
   </si>
   <si>
-    <t xml:space="preserve">Immune</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endothelial</t>
+    <t xml:space="preserve">Lymphocyte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Myeloid</t>
   </si>
   <si>
     <t xml:space="preserve">Erythroblast</t>
   </si>
   <si>
-    <t xml:space="preserve">Pericyte</t>
-  </si>
-  <si>
     <t xml:space="preserve">10X280_2_ABCD_1</t>
   </si>
   <si>
@@ -174,31 +174,28 @@
     <t xml:space="preserve">days_in_culture</t>
   </si>
   <si>
-    <t xml:space="preserve">ROBO2.Ependymal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLIT2.Ependymal</t>
-  </si>
-  <si>
     <t xml:space="preserve">Radial.Glia</t>
   </si>
   <si>
-    <t xml:space="preserve">Transit.Amplifying.Cell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAX3.Neuroblast</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAX3.Neuron</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOXB3.Neuroblast</t>
+    <t xml:space="preserve">Intermediate.Proliferative.Cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAX6..NEUROD1..Neuroblast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAX6..HOXB3..Neuroblast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fetal.Neuronal.Progenitor</t>
   </si>
   <si>
     <t xml:space="preserve">Fetal.COP</t>
   </si>
   <si>
-    <t xml:space="preserve">Early.Oligo</t>
+    <t xml:space="preserve">Early.OL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postnatal.Glial.Progenitor</t>
   </si>
   <si>
     <t xml:space="preserve">GSM4379132</t>
@@ -276,13 +273,7 @@
     <t xml:space="preserve">GSM7291256</t>
   </si>
   <si>
-    <t xml:space="preserve">Subgroup</t>
-  </si>
-  <si>
     <t xml:space="preserve">GSM7305260</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DMG</t>
   </si>
   <si>
     <t xml:space="preserve">GSM7305265</t>
@@ -699,61 +690,61 @@
         <v>22</v>
       </c>
       <c r="C2" t="n">
-        <v>168</v>
+        <v>473</v>
       </c>
       <c r="D2" t="n">
-        <v>281</v>
+        <v>1746</v>
       </c>
       <c r="E2" t="n">
-        <v>1817</v>
+        <v>47</v>
       </c>
       <c r="F2" t="n">
-        <v>1031</v>
+        <v>1664</v>
       </c>
       <c r="G2" t="n">
-        <v>473</v>
+        <v>38</v>
       </c>
       <c r="H2" t="n">
-        <v>2091</v>
+        <v>3468</v>
       </c>
       <c r="I2" t="n">
-        <v>2327</v>
+        <v>1295</v>
       </c>
       <c r="J2" t="n">
-        <v>112</v>
+        <v>42</v>
       </c>
       <c r="K2" t="n">
-        <v>362</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>38</v>
+        <v>495</v>
       </c>
       <c r="M2" t="n">
-        <v>154</v>
+        <v>10</v>
       </c>
       <c r="N2" t="n">
-        <v>93</v>
+        <v>3</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>411</v>
+        <v>192</v>
       </c>
       <c r="Q2" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="R2" t="n">
-        <v>143</v>
+        <v>42</v>
       </c>
       <c r="S2" t="n">
-        <v>198</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>351</v>
+        <v>141</v>
       </c>
       <c r="U2" t="n">
-        <v>33</v>
+        <v>438</v>
       </c>
     </row>
     <row r="3">
@@ -764,61 +755,61 @@
         <v>22</v>
       </c>
       <c r="C3" t="n">
-        <v>693</v>
+        <v>1255</v>
       </c>
       <c r="D3" t="n">
-        <v>458</v>
+        <v>4936</v>
       </c>
       <c r="E3" t="n">
-        <v>4583</v>
+        <v>148</v>
       </c>
       <c r="F3" t="n">
-        <v>1312</v>
+        <v>1729</v>
       </c>
       <c r="G3" t="n">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="H3" t="n">
-        <v>468</v>
+        <v>601</v>
       </c>
       <c r="I3" t="n">
-        <v>1678</v>
+        <v>1534</v>
       </c>
       <c r="J3" t="n">
-        <v>480</v>
+        <v>438</v>
       </c>
       <c r="K3" t="n">
-        <v>1250</v>
+        <v>6</v>
       </c>
       <c r="L3" t="n">
-        <v>55</v>
+        <v>1739</v>
       </c>
       <c r="M3" t="n">
-        <v>345</v>
+        <v>37</v>
       </c>
       <c r="N3" t="n">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="O3" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>808</v>
+        <v>1871</v>
       </c>
       <c r="Q3" t="n">
-        <v>123</v>
+        <v>923</v>
       </c>
       <c r="R3" t="n">
-        <v>2169</v>
+        <v>105</v>
       </c>
       <c r="S3" t="n">
-        <v>1896</v>
+        <v>2</v>
       </c>
       <c r="T3" t="n">
-        <v>432</v>
+        <v>2101</v>
       </c>
       <c r="U3" t="n">
-        <v>934</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4">
@@ -829,61 +820,61 @@
         <v>22</v>
       </c>
       <c r="C4" t="n">
-        <v>173</v>
+        <v>264</v>
       </c>
       <c r="D4" t="n">
-        <v>133</v>
+        <v>679</v>
       </c>
       <c r="E4" t="n">
-        <v>584</v>
+        <v>14</v>
       </c>
       <c r="F4" t="n">
-        <v>1435</v>
+        <v>2215</v>
       </c>
       <c r="G4" t="n">
+        <v>171</v>
+      </c>
+      <c r="H4" t="n">
+        <v>351</v>
+      </c>
+      <c r="I4" t="n">
+        <v>697</v>
+      </c>
+      <c r="J4" t="n">
+        <v>120</v>
+      </c>
+      <c r="K4" t="n">
+        <v>578</v>
+      </c>
+      <c r="L4" t="n">
+        <v>215</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
         <v>235</v>
       </c>
-      <c r="H4" t="n">
-        <v>298</v>
-      </c>
-      <c r="I4" t="n">
-        <v>855</v>
-      </c>
-      <c r="J4" t="n">
-        <v>173</v>
-      </c>
-      <c r="K4" t="n">
-        <v>118</v>
-      </c>
-      <c r="L4" t="n">
-        <v>601</v>
-      </c>
-      <c r="M4" t="n">
-        <v>107</v>
-      </c>
-      <c r="N4" t="n">
-        <v>52</v>
-      </c>
-      <c r="O4" t="n">
-        <v>11</v>
-      </c>
-      <c r="P4" t="n">
-        <v>540</v>
-      </c>
       <c r="Q4" t="n">
-        <v>1214</v>
+        <v>365</v>
       </c>
       <c r="R4" t="n">
-        <v>314</v>
+        <v>1172</v>
       </c>
       <c r="S4" t="n">
-        <v>222</v>
+        <v>5</v>
       </c>
       <c r="T4" t="n">
-        <v>38</v>
+        <v>311</v>
       </c>
       <c r="U4" t="n">
-        <v>337</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -894,61 +885,61 @@
         <v>22</v>
       </c>
       <c r="C5" t="n">
-        <v>408</v>
+        <v>511</v>
       </c>
       <c r="D5" t="n">
-        <v>32</v>
+        <v>583</v>
       </c>
       <c r="E5" t="n">
-        <v>633</v>
+        <v>59</v>
       </c>
       <c r="F5" t="n">
-        <v>638</v>
+        <v>746</v>
       </c>
       <c r="G5" t="n">
-        <v>2183</v>
+        <v>4513</v>
       </c>
       <c r="H5" t="n">
-        <v>1464</v>
+        <v>231</v>
       </c>
       <c r="I5" t="n">
-        <v>1800</v>
+        <v>1412</v>
       </c>
       <c r="J5" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="K5" t="n">
-        <v>101</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>148</v>
+        <v>202</v>
       </c>
       <c r="M5" t="n">
-        <v>123</v>
+        <v>4</v>
       </c>
       <c r="N5" t="n">
-        <v>214</v>
+        <v>7</v>
       </c>
       <c r="O5" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>406</v>
+        <v>267</v>
       </c>
       <c r="Q5" t="n">
-        <v>6</v>
+        <v>294</v>
       </c>
       <c r="R5" t="n">
-        <v>581</v>
+        <v>3</v>
       </c>
       <c r="S5" t="n">
-        <v>319</v>
+        <v>4</v>
       </c>
       <c r="T5" t="n">
-        <v>4</v>
+        <v>592</v>
       </c>
       <c r="U5" t="n">
-        <v>321</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -959,61 +950,61 @@
         <v>22</v>
       </c>
       <c r="C6" t="n">
-        <v>94</v>
+        <v>227</v>
       </c>
       <c r="D6" t="n">
-        <v>127</v>
+        <v>609</v>
       </c>
       <c r="E6" t="n">
-        <v>680</v>
+        <v>22</v>
       </c>
       <c r="F6" t="n">
-        <v>852</v>
+        <v>1204</v>
       </c>
       <c r="G6" t="n">
-        <v>149</v>
+        <v>40</v>
       </c>
       <c r="H6" t="n">
-        <v>1279</v>
+        <v>1618</v>
       </c>
       <c r="I6" t="n">
-        <v>1570</v>
+        <v>1289</v>
       </c>
       <c r="J6" t="n">
-        <v>2696</v>
+        <v>2737</v>
       </c>
       <c r="K6" t="n">
-        <v>313</v>
+        <v>645</v>
       </c>
       <c r="L6" t="n">
-        <v>568</v>
+        <v>420</v>
       </c>
       <c r="M6" t="n">
-        <v>107</v>
+        <v>884</v>
       </c>
       <c r="N6" t="n">
-        <v>862</v>
+        <v>70</v>
       </c>
       <c r="O6" t="n">
-        <v>128</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>296</v>
+        <v>84</v>
       </c>
       <c r="Q6" t="n">
-        <v>241</v>
+        <v>115</v>
       </c>
       <c r="R6" t="n">
-        <v>113</v>
+        <v>218</v>
       </c>
       <c r="S6" t="n">
-        <v>94</v>
+        <v>3</v>
       </c>
       <c r="T6" t="n">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="U6" t="n">
-        <v>114</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7">
@@ -1027,58 +1018,58 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>381</v>
+        <v>1174</v>
       </c>
       <c r="F7" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>648</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>791</v>
       </c>
       <c r="M7" t="n">
-        <v>128</v>
+        <v>364</v>
       </c>
       <c r="N7" t="n">
-        <v>465</v>
+        <v>4167</v>
       </c>
       <c r="O7" t="n">
-        <v>4143</v>
+        <v>1</v>
       </c>
       <c r="P7" t="n">
-        <v>680</v>
+        <v>10</v>
       </c>
       <c r="Q7" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="R7" t="n">
-        <v>1051</v>
+        <v>34</v>
       </c>
       <c r="S7" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="T7" t="n">
-        <v>1</v>
+        <v>1078</v>
       </c>
       <c r="U7" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1092,58 +1083,58 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
+        <v>77</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>47</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>151</v>
+      </c>
+      <c r="M8" t="n">
+        <v>99</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1495</v>
+      </c>
+      <c r="O8" t="n">
         <v>10</v>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" t="n">
-        <v>43</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="n">
-        <v>32</v>
-      </c>
-      <c r="K8" t="n">
-        <v>130</v>
-      </c>
-      <c r="L8" t="n">
-        <v>3</v>
-      </c>
-      <c r="M8" t="n">
-        <v>19</v>
-      </c>
-      <c r="N8" t="n">
-        <v>94</v>
-      </c>
-      <c r="O8" t="n">
-        <v>1497</v>
-      </c>
       <c r="P8" t="n">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="R8" t="n">
-        <v>116</v>
+        <v>20</v>
       </c>
       <c r="S8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>134</v>
       </c>
       <c r="U8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1157,58 +1148,58 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>139</v>
+        <v>386</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>188</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>223</v>
       </c>
       <c r="M9" t="n">
-        <v>33</v>
+        <v>353</v>
       </c>
       <c r="N9" t="n">
-        <v>368</v>
+        <v>2863</v>
       </c>
       <c r="O9" t="n">
-        <v>2838</v>
+        <v>99</v>
       </c>
       <c r="P9" t="n">
-        <v>233</v>
+        <v>18</v>
       </c>
       <c r="Q9" t="n">
         <v>6</v>
       </c>
       <c r="R9" t="n">
+        <v>5</v>
+      </c>
+      <c r="S9" t="n">
+        <v>15</v>
+      </c>
+      <c r="T9" t="n">
         <v>213</v>
       </c>
-      <c r="S9" t="n">
-        <v>18</v>
-      </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>13</v>
-      </c>
-      <c r="U9" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1222,58 +1213,58 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>153</v>
+        <v>480</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>306</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>492</v>
       </c>
       <c r="M10" t="n">
-        <v>190</v>
+        <v>299</v>
       </c>
       <c r="N10" t="n">
-        <v>222</v>
+        <v>1829</v>
       </c>
       <c r="O10" t="n">
-        <v>1951</v>
+        <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>290</v>
+        <v>9</v>
       </c>
       <c r="Q10" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="R10" t="n">
-        <v>430</v>
+        <v>3</v>
       </c>
       <c r="S10" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="T10" t="n">
-        <v>1</v>
+        <v>438</v>
       </c>
       <c r="U10" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1290,52 +1281,52 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>85</v>
+        <v>389</v>
       </c>
       <c r="F11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>135</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>154</v>
+      </c>
+      <c r="M11" t="n">
+        <v>57</v>
+      </c>
+      <c r="N11" t="n">
+        <v>2068</v>
+      </c>
+      <c r="O11" t="n">
+        <v>12</v>
+      </c>
+      <c r="P11" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>43</v>
+      </c>
+      <c r="S11" t="n">
         <v>7</v>
       </c>
-      <c r="G11" t="n">
-        <v>3</v>
-      </c>
-      <c r="H11" t="n">
-        <v>132</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>54</v>
-      </c>
-      <c r="K11" t="n">
-        <v>130</v>
-      </c>
-      <c r="L11" t="n">
-        <v>2</v>
-      </c>
-      <c r="M11" t="n">
-        <v>23</v>
-      </c>
-      <c r="N11" t="n">
-        <v>80</v>
-      </c>
-      <c r="O11" t="n">
-        <v>2041</v>
-      </c>
-      <c r="P11" t="n">
-        <v>306</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>44</v>
-      </c>
-      <c r="R11" t="n">
-        <v>339</v>
-      </c>
-      <c r="S11" t="n">
-        <v>6</v>
-      </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>374</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1352,58 +1343,58 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E12" t="n">
-        <v>256</v>
+        <v>900</v>
       </c>
       <c r="F12" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
+        <v>698</v>
+      </c>
+      <c r="M12" t="n">
+        <v>295</v>
+      </c>
+      <c r="N12" t="n">
+        <v>3171</v>
+      </c>
+      <c r="O12" t="n">
+        <v>23</v>
+      </c>
+      <c r="P12" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q12" t="n">
         <v>3</v>
       </c>
-      <c r="M12" t="n">
-        <v>72</v>
-      </c>
-      <c r="N12" t="n">
-        <v>349</v>
-      </c>
-      <c r="O12" t="n">
-        <v>3107</v>
-      </c>
-      <c r="P12" t="n">
-        <v>565</v>
-      </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>2</v>
       </c>
-      <c r="R12" t="n">
-        <v>152</v>
-      </c>
       <c r="S12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="U12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1417,13 +1408,13 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>54</v>
+        <v>380</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -1435,40 +1426,40 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="M13" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="N13" t="n">
-        <v>79</v>
+        <v>5257</v>
       </c>
       <c r="O13" t="n">
-        <v>5243</v>
+        <v>1</v>
       </c>
       <c r="P13" t="n">
-        <v>334</v>
+        <v>5</v>
       </c>
       <c r="Q13" t="n">
+        <v>13</v>
+      </c>
+      <c r="R13" t="n">
         <v>2</v>
       </c>
-      <c r="R13" t="n">
-        <v>133</v>
-      </c>
       <c r="S13" t="n">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="U13" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1482,13 +1473,13 @@
         <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>133</v>
+        <v>544</v>
       </c>
       <c r="F14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -1500,40 +1491,40 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>319</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>393</v>
       </c>
       <c r="M14" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N14" t="n">
-        <v>98</v>
+        <v>2549</v>
       </c>
       <c r="O14" t="n">
-        <v>2542</v>
+        <v>1</v>
       </c>
       <c r="P14" t="n">
-        <v>397</v>
+        <v>5</v>
       </c>
       <c r="Q14" t="n">
+        <v>4</v>
+      </c>
+      <c r="R14" t="n">
         <v>3</v>
       </c>
-      <c r="R14" t="n">
-        <v>280</v>
-      </c>
       <c r="S14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>313</v>
       </c>
       <c r="U14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1547,58 +1538,58 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
-        <v>357</v>
+        <v>998</v>
       </c>
       <c r="F15" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>656</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>822</v>
       </c>
       <c r="M15" t="n">
-        <v>155</v>
+        <v>663</v>
       </c>
       <c r="N15" t="n">
-        <v>763</v>
+        <v>5465</v>
       </c>
       <c r="O15" t="n">
-        <v>5338</v>
+        <v>71</v>
       </c>
       <c r="P15" t="n">
-        <v>642</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R15" t="n">
-        <v>821</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>797</v>
       </c>
       <c r="U15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1612,16 +1603,16 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>183</v>
+        <v>813</v>
       </c>
       <c r="F16" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>10</v>
@@ -1630,40 +1621,40 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>498</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>2</v>
+        <v>709</v>
       </c>
       <c r="M16" t="n">
-        <v>118</v>
+        <v>84</v>
       </c>
       <c r="N16" t="n">
-        <v>117</v>
+        <v>2888</v>
       </c>
       <c r="O16" t="n">
-        <v>2965</v>
+        <v>1</v>
       </c>
       <c r="P16" t="n">
-        <v>613</v>
+        <v>24</v>
       </c>
       <c r="Q16" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="R16" t="n">
-        <v>1445</v>
+        <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>1480</v>
       </c>
       <c r="U16" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1677,58 +1668,58 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>145</v>
+        <v>601</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
+        <v>9</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>80</v>
+      </c>
+      <c r="M17" t="n">
+        <v>43</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2049</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>12</v>
+      </c>
+      <c r="R17" t="n">
         <v>10</v>
       </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>28</v>
-      </c>
-      <c r="K17" t="n">
-        <v>65</v>
-      </c>
-      <c r="L17" t="n">
+      <c r="S17" t="n">
         <v>3</v>
       </c>
-      <c r="M17" t="n">
-        <v>16</v>
-      </c>
-      <c r="N17" t="n">
-        <v>70</v>
-      </c>
-      <c r="O17" t="n">
-        <v>2028</v>
-      </c>
-      <c r="P17" t="n">
-        <v>467</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>9</v>
-      </c>
-      <c r="R17" t="n">
-        <v>168</v>
-      </c>
-      <c r="S17" t="n">
-        <v>4</v>
-      </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>209</v>
       </c>
       <c r="U17" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1742,58 +1733,58 @@
         <v>15</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E18" t="n">
-        <v>220</v>
+        <v>847</v>
       </c>
       <c r="F18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>188</v>
+        <v>15</v>
       </c>
       <c r="L18" t="n">
-        <v>37</v>
+        <v>233</v>
       </c>
       <c r="M18" t="n">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="N18" t="n">
-        <v>134</v>
+        <v>6580</v>
       </c>
       <c r="O18" t="n">
-        <v>6562</v>
+        <v>1</v>
       </c>
       <c r="P18" t="n">
-        <v>629</v>
+        <v>8</v>
       </c>
       <c r="Q18" t="n">
-        <v>99</v>
+        <v>14</v>
       </c>
       <c r="R18" t="n">
-        <v>502</v>
+        <v>102</v>
       </c>
       <c r="S18" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="T18" t="n">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="U18" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1807,10 +1798,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>87</v>
+        <v>256</v>
       </c>
       <c r="F19" t="n">
         <v>1</v>
@@ -1819,46 +1810,46 @@
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>341</v>
       </c>
       <c r="M19" t="n">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="N19" t="n">
-        <v>128</v>
+        <v>2262</v>
       </c>
       <c r="O19" t="n">
-        <v>2265</v>
+        <v>1</v>
       </c>
       <c r="P19" t="n">
-        <v>188</v>
+        <v>7</v>
       </c>
       <c r="Q19" t="n">
+        <v>8</v>
+      </c>
+      <c r="R19" t="n">
+        <v>4</v>
+      </c>
+      <c r="S19" t="n">
         <v>3</v>
       </c>
-      <c r="R19" t="n">
-        <v>331</v>
-      </c>
-      <c r="S19" t="n">
-        <v>7</v>
-      </c>
       <c r="T19" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="U19" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1872,58 +1863,58 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>141</v>
+        <v>394</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>438</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>528</v>
       </c>
       <c r="M20" t="n">
-        <v>89</v>
+        <v>222</v>
       </c>
       <c r="N20" t="n">
-        <v>300</v>
+        <v>4957</v>
       </c>
       <c r="O20" t="n">
-        <v>4949</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>248</v>
+        <v>22</v>
       </c>
       <c r="Q20" t="n">
+        <v>34</v>
+      </c>
+      <c r="R20" t="n">
         <v>7</v>
       </c>
-      <c r="R20" t="n">
-        <v>993</v>
-      </c>
       <c r="S20" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="T20" t="n">
-        <v>1</v>
+        <v>1051</v>
       </c>
       <c r="U20" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1937,58 +1928,58 @@
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>108</v>
+        <v>344</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>4</v>
+        <v>185</v>
       </c>
       <c r="M21" t="n">
+        <v>203</v>
+      </c>
+      <c r="N21" t="n">
+        <v>3103</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q21" t="n">
         <v>31</v>
       </c>
-      <c r="N21" t="n">
-        <v>256</v>
-      </c>
-      <c r="O21" t="n">
-        <v>3056</v>
-      </c>
-      <c r="P21" t="n">
-        <v>227</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>23</v>
-      </c>
       <c r="R21" t="n">
-        <v>353</v>
+        <v>26</v>
       </c>
       <c r="S21" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="T21" t="n">
+        <v>367</v>
+      </c>
+      <c r="U21" t="n">
         <v>5</v>
-      </c>
-      <c r="U21" t="n">
-        <v>38</v>
       </c>
     </row>
     <row r="22">
@@ -2002,58 +1993,58 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="E22" t="n">
-        <v>53</v>
+        <v>356</v>
       </c>
       <c r="F22" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>87</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>91</v>
+      </c>
+      <c r="M22" t="n">
+        <v>165</v>
+      </c>
+      <c r="N22" t="n">
+        <v>2900</v>
+      </c>
+      <c r="O22" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>20</v>
+      </c>
+      <c r="R22" t="n">
+        <v>35</v>
+      </c>
+      <c r="S22" t="n">
+        <v>39</v>
+      </c>
+      <c r="T22" t="n">
+        <v>797</v>
+      </c>
+      <c r="U22" t="n">
         <v>3</v>
-      </c>
-      <c r="H22" t="n">
-        <v>84</v>
-      </c>
-      <c r="I22" t="n">
-        <v>2</v>
-      </c>
-      <c r="J22" t="n">
-        <v>64</v>
-      </c>
-      <c r="K22" t="n">
-        <v>70</v>
-      </c>
-      <c r="L22" t="n">
-        <v>22</v>
-      </c>
-      <c r="M22" t="n">
-        <v>18</v>
-      </c>
-      <c r="N22" t="n">
-        <v>204</v>
-      </c>
-      <c r="O22" t="n">
-        <v>3003</v>
-      </c>
-      <c r="P22" t="n">
-        <v>300</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>30</v>
-      </c>
-      <c r="R22" t="n">
-        <v>646</v>
-      </c>
-      <c r="S22" t="n">
-        <v>22</v>
-      </c>
-      <c r="T22" t="n">
-        <v>3</v>
-      </c>
-      <c r="U22" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="23">
@@ -2067,58 +2058,58 @@
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>31</v>
+        <v>148</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>21</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>10</v>
+      </c>
+      <c r="L23" t="n">
+        <v>73</v>
+      </c>
+      <c r="M23" t="n">
+        <v>45</v>
+      </c>
+      <c r="N23" t="n">
+        <v>1894</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>17</v>
+      </c>
+      <c r="R23" t="n">
+        <v>223</v>
+      </c>
+      <c r="S23" t="n">
+        <v>28</v>
+      </c>
+      <c r="T23" t="n">
+        <v>521</v>
+      </c>
+      <c r="U23" t="n">
         <v>2</v>
-      </c>
-      <c r="H23" t="n">
-        <v>19</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J23" t="n">
-        <v>36</v>
-      </c>
-      <c r="K23" t="n">
-        <v>63</v>
-      </c>
-      <c r="L23" t="n">
-        <v>15</v>
-      </c>
-      <c r="M23" t="n">
-        <v>9</v>
-      </c>
-      <c r="N23" t="n">
-        <v>73</v>
-      </c>
-      <c r="O23" t="n">
-        <v>1966</v>
-      </c>
-      <c r="P23" t="n">
-        <v>131</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>92</v>
-      </c>
-      <c r="R23" t="n">
-        <v>527</v>
-      </c>
-      <c r="S23" t="n">
-        <v>13</v>
-      </c>
-      <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="n">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2680,43 +2671,43 @@
         <v>50</v>
       </c>
       <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>55</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>56</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
         <v>57</v>
       </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
         <v>58</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>59</v>
-      </c>
-      <c r="O1" t="s">
-        <v>14</v>
       </c>
       <c r="P1" t="s">
         <v>15</v>
@@ -2739,22 +2730,22 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
         <v>60</v>
       </c>
-      <c r="B2" t="s">
-        <v>61</v>
-      </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -2766,28 +2757,28 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
@@ -2804,22 +2795,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
         <v>62</v>
       </c>
-      <c r="B3" t="s">
-        <v>63</v>
-      </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -2831,31 +2822,31 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="M3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O3" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
@@ -2869,22 +2860,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
         <v>64</v>
       </c>
-      <c r="B4" t="s">
-        <v>65</v>
-      </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
         <v>8</v>
       </c>
-      <c r="E4" t="n">
-        <v>5</v>
-      </c>
       <c r="F4" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -2896,31 +2887,31 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
@@ -2934,16 +2925,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" t="s">
         <v>66</v>
       </c>
-      <c r="B5" t="s">
-        <v>67</v>
-      </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -2958,10 +2949,10 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>684</v>
+        <v>702</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -2982,10 +2973,10 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>417</v>
+        <v>15</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>381</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -2999,58 +2990,58 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s">
         <v>68</v>
       </c>
-      <c r="B6" t="s">
-        <v>69</v>
-      </c>
       <c r="C6" t="n">
-        <v>45</v>
+        <v>246</v>
       </c>
       <c r="D6" t="n">
-        <v>181</v>
+        <v>129</v>
       </c>
       <c r="E6" t="n">
-        <v>520</v>
+        <v>422</v>
       </c>
       <c r="F6" t="n">
-        <v>802</v>
+        <v>906</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I6" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="J6" t="n">
-        <v>519</v>
+        <v>380</v>
       </c>
       <c r="K6" t="n">
-        <v>2125</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>4752</v>
       </c>
       <c r="M6" t="n">
-        <v>2568</v>
+        <v>8</v>
       </c>
       <c r="N6" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="O6" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="R6" t="n">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -3098,10 +3089,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
         <v>60</v>
-      </c>
-      <c r="B2" t="s">
-        <v>61</v>
       </c>
       <c r="C2" t="n">
         <v>292</v>
@@ -3121,10 +3112,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
         <v>62</v>
-      </c>
-      <c r="B3" t="s">
-        <v>63</v>
       </c>
       <c r="C3" t="n">
         <v>291</v>
@@ -3144,10 +3135,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
         <v>64</v>
-      </c>
-      <c r="B4" t="s">
-        <v>65</v>
       </c>
       <c r="C4" t="n">
         <v>288</v>
@@ -3167,10 +3158,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" t="s">
         <v>66</v>
-      </c>
-      <c r="B5" t="s">
-        <v>67</v>
       </c>
       <c r="C5" t="n">
         <v>1105</v>
@@ -3190,10 +3181,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s">
         <v>68</v>
-      </c>
-      <c r="B6" t="s">
-        <v>69</v>
       </c>
       <c r="C6" t="n">
         <v>5664</v>
@@ -3227,43 +3218,43 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
         <v>51</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>53</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
         <v>54</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>55</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>56</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" t="s">
         <v>57</v>
       </c>
-      <c r="I1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" t="s">
         <v>58</v>
-      </c>
-      <c r="L1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M1" t="s">
-        <v>59</v>
-      </c>
-      <c r="N1" t="s">
-        <v>14</v>
       </c>
       <c r="O1" t="s">
         <v>15</v>
@@ -3286,7 +3277,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" t="n">
         <v>2</v>
@@ -3295,7 +3286,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -3310,54 +3301,54 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="L2" t="n">
-        <v>6</v>
+        <v>138</v>
       </c>
       <c r="M2" t="n">
-        <v>173</v>
+        <v>455</v>
       </c>
       <c r="N2" t="n">
-        <v>420</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
         <v>27</v>
       </c>
-      <c r="R2" t="n">
-        <v>9</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
       <c r="T2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" t="n">
         <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>582</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -3375,42 +3366,42 @@
         <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="L3" t="n">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="M3" t="n">
-        <v>79</v>
+        <v>4893</v>
       </c>
       <c r="N3" t="n">
-        <v>4850</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>604</v>
+        <v>26</v>
       </c>
       <c r="P3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
         <v>116</v>
       </c>
-      <c r="R3" t="n">
-        <v>26</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
       <c r="T3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" t="n">
         <v>1</v>
@@ -3419,7 +3410,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>346</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -3437,51 +3428,51 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>104</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="L4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>5</v>
+        <v>4637</v>
       </c>
       <c r="N4" t="n">
-        <v>4634</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>347</v>
+        <v>3</v>
       </c>
       <c r="P4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q4" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" t="n">
-        <v>32</v>
-      </c>
       <c r="R4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="T4" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>394</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -3496,107 +3487,107 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>284</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>306</v>
       </c>
       <c r="L5" t="n">
-        <v>20</v>
+        <v>72</v>
       </c>
       <c r="M5" t="n">
-        <v>266</v>
+        <v>3593</v>
       </c>
       <c r="N5" t="n">
-        <v>3398</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>392</v>
+        <v>8</v>
       </c>
       <c r="P5" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q5" t="n">
         <v>10</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
+        <v>39</v>
+      </c>
+      <c r="S5" t="n">
         <v>173</v>
       </c>
-      <c r="R5" t="n">
-        <v>7</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
-      </c>
       <c r="T5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B6" t="n">
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>382</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>213</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="M6" t="n">
-        <v>30</v>
+        <v>2976</v>
       </c>
       <c r="N6" t="n">
-        <v>2976</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>381</v>
+        <v>29</v>
       </c>
       <c r="P6" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q6" t="n">
         <v>14</v>
       </c>
-      <c r="Q6" t="n">
-        <v>498</v>
-      </c>
       <c r="R6" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>478</v>
       </c>
       <c r="T6" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" t="n">
         <v>2</v>
@@ -3605,7 +3596,7 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -3620,45 +3611,45 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>127</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="L7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M7" t="n">
-        <v>35</v>
+        <v>5968</v>
       </c>
       <c r="N7" t="n">
-        <v>5943</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>127</v>
+        <v>1</v>
       </c>
       <c r="P7" t="n">
         <v>8</v>
       </c>
       <c r="Q7" t="n">
-        <v>254</v>
+        <v>8</v>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>247</v>
       </c>
       <c r="T7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" t="n">
         <v>1</v>
@@ -3667,7 +3658,7 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -3682,45 +3673,45 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>115</v>
+      </c>
+      <c r="L8" t="n">
+        <v>12</v>
+      </c>
+      <c r="M8" t="n">
+        <v>5208</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>11</v>
       </c>
-      <c r="J8" t="n">
-        <v>115</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>39</v>
-      </c>
-      <c r="N8" t="n">
-        <v>5176</v>
-      </c>
-      <c r="O8" t="n">
-        <v>181</v>
-      </c>
       <c r="P8" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q8" t="n">
         <v>6</v>
       </c>
-      <c r="Q8" t="n">
-        <v>132</v>
-      </c>
       <c r="R8" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="T8" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -3729,7 +3720,7 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -3744,54 +3735,54 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L9" t="n">
         <v>2</v>
       </c>
       <c r="M9" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N9" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
+        <v>22</v>
+      </c>
+      <c r="P9" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
         <v>2</v>
       </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>22</v>
-      </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -3800,51 +3791,51 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J10" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="L10" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="M10" t="n">
-        <v>94</v>
+        <v>280</v>
       </c>
       <c r="N10" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>152</v>
+        <v>43</v>
       </c>
       <c r="P10" t="n">
         <v>5</v>
       </c>
       <c r="Q10" t="n">
+        <v>6</v>
+      </c>
+      <c r="R10" t="n">
+        <v>5</v>
+      </c>
+      <c r="S10" t="n">
         <v>46</v>
       </c>
-      <c r="R10" t="n">
-        <v>43</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
       <c r="T10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B11" t="n">
         <v>1</v>
@@ -3853,7 +3844,7 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -3868,45 +3859,45 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>153</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="L11" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="M11" t="n">
-        <v>16</v>
+        <v>2284</v>
       </c>
       <c r="N11" t="n">
-        <v>2279</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="P11" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q11" t="n">
         <v>4</v>
       </c>
-      <c r="Q11" t="n">
-        <v>57</v>
-      </c>
       <c r="R11" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="T11" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" t="n">
         <v>23</v>
@@ -3915,7 +3906,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>131</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -3924,51 +3915,51 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>20</v>
+      </c>
+      <c r="L12" t="n">
+        <v>13</v>
+      </c>
+      <c r="M12" t="n">
+        <v>571</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>27</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>4</v>
+      </c>
+      <c r="R12" t="n">
         <v>9</v>
       </c>
-      <c r="J12" t="n">
-        <v>14</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>4</v>
-      </c>
-      <c r="M12" t="n">
-        <v>40</v>
-      </c>
-      <c r="N12" t="n">
-        <v>539</v>
-      </c>
-      <c r="O12" t="n">
-        <v>138</v>
-      </c>
-      <c r="P12" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>18</v>
-      </c>
-      <c r="R12" t="n">
-        <v>27</v>
-      </c>
       <c r="S12" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="T12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" t="n">
         <v>9</v>
@@ -3977,7 +3968,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>265</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -3992,54 +3983,54 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>17</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M13" t="n">
+        <v>373</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>15</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>7</v>
+      </c>
+      <c r="R13" t="n">
         <v>23</v>
       </c>
-      <c r="J13" t="n">
-        <v>12</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>5</v>
-      </c>
-      <c r="M13" t="n">
-        <v>10</v>
-      </c>
-      <c r="N13" t="n">
-        <v>366</v>
-      </c>
-      <c r="O13" t="n">
-        <v>266</v>
-      </c>
-      <c r="P13" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>86</v>
-      </c>
-      <c r="R13" t="n">
-        <v>14</v>
-      </c>
       <c r="S13" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="T13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" t="n">
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -4054,37 +4045,37 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="L14" t="n">
         <v>7</v>
       </c>
       <c r="M14" t="n">
+        <v>4195</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
         <v>9</v>
       </c>
-      <c r="N14" t="n">
-        <v>4185</v>
-      </c>
-      <c r="O14" t="n">
-        <v>71</v>
-      </c>
       <c r="P14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="R14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -4092,78 +4083,78 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" t="n">
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>13</v>
+        <v>852</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="L15" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="M15" t="n">
-        <v>69</v>
+        <v>6167</v>
       </c>
       <c r="N15" t="n">
-        <v>6116</v>
+        <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>847</v>
+        <v>70</v>
       </c>
       <c r="P15" t="n">
-        <v>83</v>
+        <v>51</v>
       </c>
       <c r="Q15" t="n">
-        <v>845</v>
+        <v>84</v>
       </c>
       <c r="R15" t="n">
-        <v>71</v>
+        <v>113</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>827</v>
       </c>
       <c r="T15" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>130</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -4178,40 +4169,40 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>131</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="L16" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M16" t="n">
-        <v>21</v>
+        <v>1648</v>
       </c>
       <c r="N16" t="n">
-        <v>1638</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="P16" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q16" t="n">
         <v>4</v>
       </c>
-      <c r="Q16" t="n">
-        <v>95</v>
-      </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="S16" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="T16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4247,7 +4238,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" t="n">
         <v>12</v>
@@ -4267,7 +4258,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" t="n">
         <v>27</v>
@@ -4287,7 +4278,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" t="n">
         <v>2</v>
@@ -4307,7 +4298,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" t="n">
         <v>28</v>
@@ -4327,7 +4318,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B6" t="n">
         <v>12</v>
@@ -4347,7 +4338,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" t="n">
         <v>6</v>
@@ -4367,7 +4358,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" t="n">
         <v>12</v>
@@ -4387,7 +4378,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" t="n">
         <v>4</v>
@@ -4407,7 +4398,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" t="n">
         <v>31</v>
@@ -4427,7 +4418,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B11" t="n">
         <v>18</v>
@@ -4447,7 +4438,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" t="n">
         <v>29</v>
@@ -4467,7 +4458,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" t="n">
         <v>6</v>
@@ -4487,7 +4478,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" t="n">
         <v>18</v>
@@ -4507,7 +4498,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" t="n">
         <v>43</v>
@@ -4527,7 +4518,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B16" t="n">
         <v>3</v>
@@ -4561,454 +4552,412 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>85</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="M1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="O1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="P1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="R1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="S1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" t="s">
-        <v>87</v>
+        <v>84</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
-        <v>110</v>
+        <v>396</v>
       </c>
       <c r="F2" t="n">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>7</v>
+        <v>1324</v>
       </c>
       <c r="H2" t="n">
-        <v>1160</v>
+        <v>85</v>
       </c>
       <c r="I2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
-        <v>218</v>
+        <v>5496</v>
       </c>
       <c r="K2" t="n">
-        <v>4086</v>
+        <v>137</v>
       </c>
       <c r="L2" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="M2" t="n">
-        <v>1366</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>257</v>
+        <v>5</v>
       </c>
       <c r="O2" t="n">
-        <v>209</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="R2" t="n">
-        <v>848</v>
+        <v>751</v>
       </c>
       <c r="S2" t="n">
-        <v>5</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B3" t="s">
-        <v>87</v>
+        <v>85</v>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>93</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="E3" t="n">
-        <v>218</v>
+        <v>464</v>
       </c>
       <c r="F3" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="H3" t="n">
-        <v>54</v>
+        <v>349</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>462</v>
+        <v>3616</v>
       </c>
       <c r="K3" t="n">
-        <v>1876</v>
+        <v>93</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M3" t="n">
-        <v>1381</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>236</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>411</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="R3" t="n">
-        <v>260</v>
+        <v>53</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B4" t="s">
-        <v>87</v>
+        <v>86</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>257</v>
       </c>
       <c r="F4" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
+        <v>90</v>
+      </c>
+      <c r="H4" t="n">
+        <v>342</v>
+      </c>
+      <c r="I4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1499</v>
+      </c>
+      <c r="K4" t="n">
+        <v>155</v>
+      </c>
+      <c r="L4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" t="n">
         <v>8</v>
       </c>
-      <c r="H4" t="n">
-        <v>134</v>
-      </c>
-      <c r="I4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J4" t="n">
-        <v>833</v>
-      </c>
-      <c r="K4" t="n">
-        <v>341</v>
-      </c>
-      <c r="L4" t="n">
-        <v>43</v>
-      </c>
-      <c r="M4" t="n">
-        <v>111</v>
-      </c>
       <c r="N4" t="n">
-        <v>291</v>
+        <v>28</v>
       </c>
       <c r="O4" t="n">
-        <v>997</v>
+        <v>3</v>
       </c>
       <c r="P4" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="Q4" t="n">
-        <v>3</v>
+        <v>1027</v>
       </c>
       <c r="R4" t="n">
-        <v>2151</v>
+        <v>1457</v>
       </c>
       <c r="S4" t="n">
-        <v>13</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B5" t="s">
         <v>87</v>
       </c>
+      <c r="B5" t="n">
+        <v>11</v>
+      </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>281</v>
       </c>
       <c r="D5" t="n">
+        <v>101</v>
+      </c>
+      <c r="E5" t="n">
+        <v>700</v>
+      </c>
+      <c r="F5" t="n">
         <v>3</v>
       </c>
-      <c r="E5" t="n">
-        <v>240</v>
-      </c>
-      <c r="F5" t="n">
-        <v>290</v>
-      </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="H5" t="n">
-        <v>115</v>
+        <v>1040</v>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1413</v>
+        <v>692</v>
       </c>
       <c r="K5" t="n">
-        <v>487</v>
+        <v>116</v>
       </c>
       <c r="L5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="M5" t="n">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>242</v>
+        <v>2</v>
       </c>
       <c r="O5" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>380</v>
       </c>
       <c r="R5" t="n">
-        <v>1074</v>
+        <v>785</v>
       </c>
       <c r="S5" t="n">
-        <v>3</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B6" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>174</v>
+        <v>63</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="L6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N6" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="R6" t="n">
-        <v>703</v>
+        <v>422</v>
       </c>
       <c r="S6" t="n">
         <v>4</v>
       </c>
-      <c r="T6" t="n">
-        <v>4</v>
-      </c>
-      <c r="U6" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="E7" t="n">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="F7" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="H7" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7" t="n">
-        <v>16</v>
+        <v>878</v>
       </c>
       <c r="K7" t="n">
-        <v>396</v>
+        <v>82</v>
       </c>
       <c r="L7" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="M7" t="n">
-        <v>374</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>283</v>
+        <v>2</v>
       </c>
       <c r="O7" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P7" t="n">
-        <v>463</v>
+        <v>175</v>
       </c>
       <c r="Q7" t="n">
-        <v>103</v>
+        <v>1</v>
       </c>
       <c r="R7" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="S7" t="n">
-        <v>3</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5027,160 +4976,139 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" t="s">
-        <v>87</v>
+        <v>84</v>
+      </c>
+      <c r="B2" t="n">
+        <v>7173</v>
       </c>
       <c r="C2" t="n">
-        <v>6998</v>
+        <v>753</v>
       </c>
       <c r="D2" t="n">
-        <v>719</v>
+        <v>257</v>
       </c>
       <c r="E2" t="n">
-        <v>400</v>
+        <v>21</v>
       </c>
       <c r="F2" t="n">
-        <v>120</v>
-      </c>
-      <c r="G2" t="n">
-        <v>247</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B3" t="s">
-        <v>87</v>
+        <v>85</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3567</v>
       </c>
       <c r="C3" t="n">
-        <v>3642</v>
+        <v>567</v>
       </c>
       <c r="D3" t="n">
-        <v>470</v>
+        <v>786</v>
       </c>
       <c r="E3" t="n">
-        <v>752</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>46</v>
-      </c>
-      <c r="G3" t="n">
-        <v>96</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B4" t="s">
-        <v>87</v>
+        <v>86</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3372</v>
       </c>
       <c r="C4" t="n">
-        <v>3281</v>
+        <v>134</v>
       </c>
       <c r="D4" t="n">
-        <v>134</v>
+        <v>721</v>
       </c>
       <c r="E4" t="n">
-        <v>710</v>
+        <v>83</v>
       </c>
       <c r="F4" t="n">
-        <v>133</v>
-      </c>
-      <c r="G4" t="n">
-        <v>740</v>
+        <v>688</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B5" t="s">
         <v>87</v>
       </c>
+      <c r="B5" t="n">
+        <v>3361</v>
+      </c>
       <c r="C5" t="n">
-        <v>3254</v>
+        <v>43</v>
       </c>
       <c r="D5" t="n">
-        <v>53</v>
+        <v>265</v>
       </c>
       <c r="E5" t="n">
-        <v>310</v>
+        <v>65</v>
       </c>
       <c r="F5" t="n">
-        <v>44</v>
-      </c>
-      <c r="G5" t="n">
-        <v>534</v>
+        <v>461</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B6" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+      <c r="B6" t="n">
+        <v>353</v>
       </c>
       <c r="C6" t="n">
-        <v>360</v>
+        <v>48</v>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>385</v>
       </c>
       <c r="E6" t="n">
-        <v>361</v>
+        <v>27</v>
       </c>
       <c r="F6" t="n">
-        <v>54</v>
-      </c>
-      <c r="G6" t="n">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="B7" t="n">
+        <v>475</v>
       </c>
       <c r="C7" t="n">
-        <v>600</v>
+        <v>23</v>
       </c>
       <c r="D7" t="n">
-        <v>70</v>
+        <v>859</v>
       </c>
       <c r="E7" t="n">
-        <v>708</v>
+        <v>44</v>
       </c>
       <c r="F7" t="n">
-        <v>54</v>
-      </c>
-      <c r="G7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>

</xml_diff>